<commit_message>
List of currencies by default settings
</commit_message>
<xml_diff>
--- a/config/list_currencies.xlsx
+++ b/config/list_currencies.xlsx
@@ -25,10 +25,10 @@
     <t>GBP</t>
   </si>
   <si>
-    <t>AUD</t>
+    <t>currencies</t>
   </si>
   <si>
-    <t>currencies</t>
+    <t>UAH</t>
   </si>
 </sst>
 </file>
@@ -388,7 +388,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -408,7 +408,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>